<commit_message>
Templates: signed amounts for FB50, FB01, FBS1, FB60, FB65, FB70, FB75 (BAPI_ACC_DOCUMENT_POST takes direction from the amount sign); VK11 via recording, not BAPI_PRICES_CONDITIONS; overlap rules corrected; no 'fictional' labels
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finance-controlling/ABZON-asset-acquisition.xlsx
+++ b/finance-controlling/ABZON-asset-acquisition.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24a7865e3124cb3d/Documents/PostNow/github-templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24a7865e3124cb3d/Documents/PostNow/github-templates/finance-controlling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_C5ADC2FD48FB3D1BDA0814AFE865F60D2B8650A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99753713-9E06-47B0-95BD-663115F3152C}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="11_C5ADC2FD48FB3D1BDA0814AFE865F60D2B8650A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83B22C3D-9B4C-4635-901F-AFDED2F4F770}"/>
   <bookViews>
-    <workbookView xWindow="3820" yWindow="3110" windowWidth="11610" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="5" r:id="rId1"/>
@@ -1272,9 +1272,6 @@
     <t>Start your 14 day free trial at postnow.ai</t>
   </si>
   <si>
-    <t>Template provided free by PostNow.ai. All sample data is fictional. Validate field requirements against your own configuration before a production load.</t>
-  </si>
-  <si>
     <t>Asset Acquisition with Automatic Offsetting Entry</t>
   </si>
   <si>
@@ -1296,7 +1293,10 @@
     <t>https://postnow.ai/templates/finance-controlling</t>
   </si>
   <si>
-    <t>Sheets: Template (enter your data), Field Guide, BAPI Mapping, How It Works. Mandatory columns have a dark green heading and an asterisk. Sample data is fictional.</t>
+    <t>Sheets: Template (enter your data), Field Guide, BAPI Mapping, How It Works. Mandatory columns have a dark green heading and an asterisk.</t>
+  </si>
+  <si>
+    <t>Template provided free by PostNow.ai. Validate field requirements against your own configuration before a production load.</t>
   </si>
 </sst>
 </file>
@@ -1316,11 +1316,13 @@
       <sz val="18"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFD9EAE0"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1328,110 +1330,129 @@
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF5B6B62"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF0F2E1D"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF1A1A1A"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF14532D"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF1A1A1A"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF1E8E4E"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0F2E1D"/>
       <name val="Consolas"/>
+      <family val="3"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF14532D"/>
       <name val="Consolas"/>
+      <family val="3"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFB45309"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="26"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color rgb="FFCFE8DA"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF1A1A1A"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF5B6B62"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF14532D"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="10"/>
       <color rgb="FF1155CC"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF14532D"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1439,6 +1460,7 @@
       <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -1606,6 +1628,11 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
@@ -1625,6 +1652,9 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
@@ -1632,28 +1662,10 @@
     <xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1662,14 +1674,24 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2118,6 +2140,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2407,47 +2433,47 @@
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="3.6328125" customWidth="1"/>
-    <col min="2" max="2" width="30.6328125" style="46" customWidth="1"/>
-    <col min="3" max="3" width="70.6328125" style="46" customWidth="1"/>
+    <col min="2" max="2" width="30.6328125" style="25" customWidth="1"/>
+    <col min="3" max="3" width="70.6328125" style="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:3" ht="26" x14ac:dyDescent="0.65">
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="22" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B4" s="23" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B4" s="44" t="s">
+      <c r="C4" s="25" t="s">
         <v>278</v>
       </c>
-      <c r="C4" s="46" t="s">
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B5" s="23" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B5" s="44" t="s">
+      <c r="C5" s="25" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B7" s="24" t="s">
         <v>280</v>
       </c>
-      <c r="C5" s="46" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B7" s="45" t="s">
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B8" s="23" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B8" s="44" t="s">
+      <c r="C8" s="26" t="s">
         <v>282</v>
       </c>
-      <c r="C8" s="47" t="s">
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B10" s="23" t="s">
         <v>283</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B10" s="44" t="s">
-        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -2491,124 +2517,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="28"/>
+      <c r="S1" s="28"/>
+      <c r="T1" s="28"/>
+      <c r="U1" s="28"/>
+      <c r="V1" s="28"/>
+      <c r="W1" s="28"/>
+      <c r="X1" s="28"/>
+      <c r="Y1" s="28"/>
+      <c r="Z1" s="28"/>
     </row>
     <row r="2" spans="1:26" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="23"/>
-      <c r="Z2" s="23"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+      <c r="P2" s="28"/>
+      <c r="Q2" s="28"/>
+      <c r="R2" s="28"/>
+      <c r="S2" s="28"/>
+      <c r="T2" s="28"/>
+      <c r="U2" s="28"/>
+      <c r="V2" s="28"/>
+      <c r="W2" s="28"/>
+      <c r="X2" s="28"/>
+      <c r="Y2" s="28"/>
+      <c r="Z2" s="28"/>
     </row>
     <row r="3" spans="1:26" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="23"/>
-      <c r="I3" s="23"/>
-      <c r="J3" s="23"/>
-      <c r="K3" s="23"/>
-      <c r="L3" s="23"/>
-      <c r="M3" s="23"/>
-      <c r="N3" s="23"/>
-      <c r="O3" s="23"/>
-      <c r="P3" s="23"/>
-      <c r="Q3" s="23"/>
-      <c r="R3" s="23"/>
-      <c r="S3" s="23"/>
-      <c r="T3" s="23"/>
-      <c r="U3" s="23"/>
-      <c r="V3" s="23"/>
-      <c r="W3" s="23"/>
-      <c r="X3" s="23"/>
-      <c r="Y3" s="23"/>
-      <c r="Z3" s="23"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="28"/>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="28"/>
+      <c r="R3" s="28"/>
+      <c r="S3" s="28"/>
+      <c r="T3" s="28"/>
+      <c r="U3" s="28"/>
+      <c r="V3" s="28"/>
+      <c r="W3" s="28"/>
+      <c r="X3" s="28"/>
+      <c r="Y3" s="28"/>
+      <c r="Z3" s="28"/>
     </row>
     <row r="4" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23"/>
-      <c r="R4" s="23"/>
-      <c r="S4" s="23"/>
-      <c r="T4" s="23"/>
-      <c r="U4" s="23"/>
-      <c r="V4" s="23"/>
-      <c r="W4" s="23"/>
-      <c r="X4" s="23"/>
-      <c r="Y4" s="23"/>
-      <c r="Z4" s="23"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="28"/>
+      <c r="N4" s="28"/>
+      <c r="O4" s="28"/>
+      <c r="P4" s="28"/>
+      <c r="Q4" s="28"/>
+      <c r="R4" s="28"/>
+      <c r="S4" s="28"/>
+      <c r="T4" s="28"/>
+      <c r="U4" s="28"/>
+      <c r="V4" s="28"/>
+      <c r="W4" s="28"/>
+      <c r="X4" s="28"/>
+      <c r="Y4" s="28"/>
+      <c r="Z4" s="28"/>
     </row>
     <row r="5" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
@@ -3114,67 +3140,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="27" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
     </row>
     <row r="2" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
     </row>
     <row r="4" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="32" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
     </row>
     <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="32" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
     </row>
     <row r="9" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="33" t="s">
         <v>94</v>
       </c>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
     </row>
     <row r="10" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
@@ -3572,67 +3598,67 @@
       <c r="E36" s="16"/>
     </row>
     <row r="38" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="28" t="s">
+      <c r="A38" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="B38" s="23"/>
-      <c r="C38" s="23"/>
-      <c r="D38" s="23"/>
-      <c r="E38" s="23"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="28"/>
     </row>
     <row r="39" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="27" t="s">
+      <c r="A39" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="B39" s="23"/>
-      <c r="C39" s="23"/>
-      <c r="D39" s="23"/>
-      <c r="E39" s="23"/>
+      <c r="B39" s="28"/>
+      <c r="C39" s="28"/>
+      <c r="D39" s="28"/>
+      <c r="E39" s="28"/>
     </row>
     <row r="40" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="27" t="s">
+      <c r="A40" s="32" t="s">
         <v>152</v>
       </c>
-      <c r="B40" s="23"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="23"/>
-      <c r="E40" s="23"/>
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
     </row>
     <row r="41" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="27" t="s">
+      <c r="A41" s="32" t="s">
         <v>153</v>
       </c>
-      <c r="B41" s="23"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="23"/>
-      <c r="E41" s="23"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="28"/>
     </row>
     <row r="42" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="27" t="s">
+      <c r="A42" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="B42" s="23"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="23"/>
-      <c r="E42" s="23"/>
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
     </row>
     <row r="43" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="27" t="s">
+      <c r="A43" s="32" t="s">
         <v>155</v>
       </c>
-      <c r="B43" s="23"/>
-      <c r="C43" s="23"/>
-      <c r="D43" s="23"/>
-      <c r="E43" s="23"/>
+      <c r="B43" s="28"/>
+      <c r="C43" s="28"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="28"/>
     </row>
     <row r="44" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="27" t="s">
+      <c r="A44" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B44" s="23"/>
-      <c r="C44" s="23"/>
-      <c r="D44" s="23"/>
-      <c r="E44" s="23"/>
+      <c r="B44" s="28"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -3669,104 +3695,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="27" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
     </row>
     <row r="2" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="31" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
     </row>
     <row r="4" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="33" t="s">
         <v>159</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="32" t="s">
         <v>161</v>
       </c>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>162</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="32" t="s">
         <v>163</v>
       </c>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
     </row>
     <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>164</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
     </row>
     <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="32" t="s">
         <v>167</v>
       </c>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>168</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="32" t="s">
         <v>169</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
     </row>
     <row r="11" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="37" t="s">
         <v>170</v>
       </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
     </row>
     <row r="13" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="28" t="s">
+      <c r="A13" s="33" t="s">
         <v>171</v>
       </c>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
     </row>
     <row r="14" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
@@ -4150,80 +4176,81 @@
       <c r="E40" s="16"/>
     </row>
     <row r="42" spans="1:5" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="28" t="s">
+      <c r="A42" s="33" t="s">
         <v>209</v>
       </c>
-      <c r="B42" s="23"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="23"/>
-      <c r="E42" s="23"/>
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
     </row>
     <row r="43" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="B43" s="29" t="s">
+      <c r="B43" s="35" t="s">
         <v>211</v>
       </c>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
-      <c r="E43" s="30"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="36"/>
+      <c r="E43" s="36"/>
     </row>
     <row r="44" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="20" t="s">
         <v>212</v>
       </c>
-      <c r="B44" s="29" t="s">
+      <c r="B44" s="35" t="s">
         <v>213</v>
       </c>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="30"/>
+      <c r="C44" s="36"/>
+      <c r="D44" s="36"/>
+      <c r="E44" s="36"/>
     </row>
     <row r="45" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="20" t="s">
         <v>214</v>
       </c>
-      <c r="B45" s="29" t="s">
+      <c r="B45" s="35" t="s">
         <v>215</v>
       </c>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
-      <c r="E45" s="30"/>
+      <c r="C45" s="36"/>
+      <c r="D45" s="36"/>
+      <c r="E45" s="36"/>
     </row>
     <row r="46" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="20" t="s">
         <v>216</v>
       </c>
-      <c r="B46" s="29" t="s">
+      <c r="B46" s="35" t="s">
         <v>217</v>
       </c>
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
-      <c r="E46" s="30"/>
+      <c r="C46" s="36"/>
+      <c r="D46" s="36"/>
+      <c r="E46" s="36"/>
     </row>
     <row r="47" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="B47" s="29" t="s">
+      <c r="B47" s="35" t="s">
         <v>219</v>
       </c>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
-      <c r="E47" s="30"/>
+      <c r="C47" s="36"/>
+      <c r="D47" s="36"/>
+      <c r="E47" s="36"/>
     </row>
     <row r="49" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="32" t="s">
+      <c r="A49" s="34" t="s">
         <v>220</v>
       </c>
-      <c r="B49" s="23"/>
-      <c r="C49" s="23"/>
-      <c r="D49" s="23"/>
-      <c r="E49" s="23"/>
+      <c r="B49" s="28"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A49:E49"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="A1:E1"/>
@@ -4240,7 +4267,6 @@
     <mergeCell ref="A42:E42"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B44:E44"/>
-    <mergeCell ref="A11:E11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4268,203 +4294,203 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="44" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="45" t="s">
         <v>221</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
     </row>
     <row r="2" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="41" t="s">
         <v>222</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
     </row>
     <row r="3" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="46" t="s">
         <v>223</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="23"/>
-      <c r="I3" s="23"/>
-      <c r="J3" s="23"/>
-      <c r="K3" s="23"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="28"/>
     </row>
     <row r="4" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="23"/>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
+      <c r="A4" s="28"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="28"/>
     </row>
     <row r="5" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="7" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="9" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="42" t="s">
+      <c r="A9" s="44" t="s">
         <v>224</v>
       </c>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="28"/>
+      <c r="K9" s="28"/>
     </row>
     <row r="11" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="28" t="s">
+      <c r="A11" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="23"/>
-      <c r="K11" s="23"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="28"/>
     </row>
     <row r="12" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C12" s="39" t="s">
+      <c r="C12" s="43" t="s">
         <v>226</v>
       </c>
-      <c r="D12" s="30"/>
-      <c r="E12" s="36" t="s">
+      <c r="D12" s="36"/>
+      <c r="E12" s="42" t="s">
         <v>227</v>
       </c>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="35" t="s">
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="47" t="s">
         <v>228</v>
       </c>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
-      <c r="K12" s="30"/>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="36"/>
     </row>
     <row r="13" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C13" s="39" t="s">
+      <c r="C13" s="43" t="s">
         <v>229</v>
       </c>
-      <c r="D13" s="30"/>
-      <c r="E13" s="36" t="s">
+      <c r="D13" s="36"/>
+      <c r="E13" s="42" t="s">
         <v>230</v>
       </c>
-      <c r="F13" s="30"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="35" t="s">
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="47" t="s">
         <v>231</v>
       </c>
-      <c r="I13" s="30"/>
-      <c r="J13" s="30"/>
-      <c r="K13" s="30"/>
+      <c r="I13" s="36"/>
+      <c r="J13" s="36"/>
+      <c r="K13" s="36"/>
     </row>
     <row r="15" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="33" t="s">
         <v>232</v>
       </c>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="28"/>
+      <c r="K15" s="28"/>
     </row>
     <row r="16" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="21">
         <v>1</v>
       </c>
-      <c r="C16" s="33" t="s">
+      <c r="C16" s="39" t="s">
         <v>233</v>
       </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="28"/>
+      <c r="K16" s="28"/>
     </row>
     <row r="17" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="32" t="s">
         <v>234</v>
       </c>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="23"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="28"/>
+      <c r="K17" s="28"/>
     </row>
     <row r="19" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="21">
         <v>2</v>
       </c>
-      <c r="C19" s="33" t="s">
+      <c r="C19" s="39" t="s">
         <v>235</v>
       </c>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="28"/>
+      <c r="K19" s="28"/>
     </row>
     <row r="20" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C20" s="27" t="s">
+      <c r="C20" s="32" t="s">
         <v>236</v>
       </c>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="23"/>
-      <c r="K20" s="23"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="28"/>
+      <c r="J20" s="28"/>
+      <c r="K20" s="28"/>
     </row>
     <row r="21" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="22" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -4486,46 +4512,46 @@
     <row r="38" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="39" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="40" spans="2:11" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C40" s="34" t="s">
+      <c r="C40" s="38" t="s">
         <v>237</v>
       </c>
-      <c r="D40" s="23"/>
-      <c r="E40" s="23"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
-      <c r="H40" s="23"/>
-      <c r="I40" s="23"/>
-      <c r="J40" s="23"/>
-      <c r="K40" s="23"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="28"/>
+      <c r="I40" s="28"/>
+      <c r="J40" s="28"/>
+      <c r="K40" s="28"/>
     </row>
     <row r="42" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="21">
         <v>3</v>
       </c>
-      <c r="C42" s="33" t="s">
+      <c r="C42" s="39" t="s">
         <v>238</v>
       </c>
-      <c r="D42" s="23"/>
-      <c r="E42" s="23"/>
-      <c r="F42" s="23"/>
-      <c r="G42" s="23"/>
-      <c r="H42" s="23"/>
-      <c r="I42" s="23"/>
-      <c r="J42" s="23"/>
-      <c r="K42" s="23"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="28"/>
+      <c r="F42" s="28"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="28"/>
+      <c r="I42" s="28"/>
+      <c r="J42" s="28"/>
+      <c r="K42" s="28"/>
     </row>
     <row r="43" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C43" s="27" t="s">
+      <c r="C43" s="32" t="s">
         <v>239</v>
       </c>
-      <c r="D43" s="23"/>
-      <c r="E43" s="23"/>
-      <c r="F43" s="23"/>
-      <c r="G43" s="23"/>
-      <c r="H43" s="23"/>
-      <c r="I43" s="23"/>
-      <c r="J43" s="23"/>
-      <c r="K43" s="23"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="28"/>
+      <c r="F43" s="28"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="28"/>
+      <c r="I43" s="28"/>
+      <c r="J43" s="28"/>
+      <c r="K43" s="28"/>
     </row>
     <row r="44" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="45" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -4552,46 +4578,46 @@
     <row r="66" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="67" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="68" spans="2:11" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C68" s="34" t="s">
+      <c r="C68" s="38" t="s">
         <v>240</v>
       </c>
-      <c r="D68" s="23"/>
-      <c r="E68" s="23"/>
-      <c r="F68" s="23"/>
-      <c r="G68" s="23"/>
-      <c r="H68" s="23"/>
-      <c r="I68" s="23"/>
-      <c r="J68" s="23"/>
-      <c r="K68" s="23"/>
+      <c r="D68" s="28"/>
+      <c r="E68" s="28"/>
+      <c r="F68" s="28"/>
+      <c r="G68" s="28"/>
+      <c r="H68" s="28"/>
+      <c r="I68" s="28"/>
+      <c r="J68" s="28"/>
+      <c r="K68" s="28"/>
     </row>
     <row r="70" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B70" s="21">
         <v>4</v>
       </c>
-      <c r="C70" s="33" t="s">
+      <c r="C70" s="39" t="s">
         <v>241</v>
       </c>
-      <c r="D70" s="23"/>
-      <c r="E70" s="23"/>
-      <c r="F70" s="23"/>
-      <c r="G70" s="23"/>
-      <c r="H70" s="23"/>
-      <c r="I70" s="23"/>
-      <c r="J70" s="23"/>
-      <c r="K70" s="23"/>
+      <c r="D70" s="28"/>
+      <c r="E70" s="28"/>
+      <c r="F70" s="28"/>
+      <c r="G70" s="28"/>
+      <c r="H70" s="28"/>
+      <c r="I70" s="28"/>
+      <c r="J70" s="28"/>
+      <c r="K70" s="28"/>
     </row>
     <row r="71" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C71" s="27" t="s">
+      <c r="C71" s="32" t="s">
         <v>242</v>
       </c>
-      <c r="D71" s="23"/>
-      <c r="E71" s="23"/>
-      <c r="F71" s="23"/>
-      <c r="G71" s="23"/>
-      <c r="H71" s="23"/>
-      <c r="I71" s="23"/>
-      <c r="J71" s="23"/>
-      <c r="K71" s="23"/>
+      <c r="D71" s="28"/>
+      <c r="E71" s="28"/>
+      <c r="F71" s="28"/>
+      <c r="G71" s="28"/>
+      <c r="H71" s="28"/>
+      <c r="I71" s="28"/>
+      <c r="J71" s="28"/>
+      <c r="K71" s="28"/>
     </row>
     <row r="72" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="73" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -4618,46 +4644,46 @@
     <row r="94" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="95" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="96" spans="3:11" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C96" s="34" t="s">
+      <c r="C96" s="38" t="s">
         <v>243</v>
       </c>
-      <c r="D96" s="23"/>
-      <c r="E96" s="23"/>
-      <c r="F96" s="23"/>
-      <c r="G96" s="23"/>
-      <c r="H96" s="23"/>
-      <c r="I96" s="23"/>
-      <c r="J96" s="23"/>
-      <c r="K96" s="23"/>
+      <c r="D96" s="28"/>
+      <c r="E96" s="28"/>
+      <c r="F96" s="28"/>
+      <c r="G96" s="28"/>
+      <c r="H96" s="28"/>
+      <c r="I96" s="28"/>
+      <c r="J96" s="28"/>
+      <c r="K96" s="28"/>
     </row>
     <row r="98" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B98" s="21">
         <v>5</v>
       </c>
-      <c r="C98" s="33" t="s">
+      <c r="C98" s="39" t="s">
         <v>244</v>
       </c>
-      <c r="D98" s="23"/>
-      <c r="E98" s="23"/>
-      <c r="F98" s="23"/>
-      <c r="G98" s="23"/>
-      <c r="H98" s="23"/>
-      <c r="I98" s="23"/>
-      <c r="J98" s="23"/>
-      <c r="K98" s="23"/>
+      <c r="D98" s="28"/>
+      <c r="E98" s="28"/>
+      <c r="F98" s="28"/>
+      <c r="G98" s="28"/>
+      <c r="H98" s="28"/>
+      <c r="I98" s="28"/>
+      <c r="J98" s="28"/>
+      <c r="K98" s="28"/>
     </row>
     <row r="99" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C99" s="27" t="s">
+      <c r="C99" s="32" t="s">
         <v>245</v>
       </c>
-      <c r="D99" s="23"/>
-      <c r="E99" s="23"/>
-      <c r="F99" s="23"/>
-      <c r="G99" s="23"/>
-      <c r="H99" s="23"/>
-      <c r="I99" s="23"/>
-      <c r="J99" s="23"/>
-      <c r="K99" s="23"/>
+      <c r="D99" s="28"/>
+      <c r="E99" s="28"/>
+      <c r="F99" s="28"/>
+      <c r="G99" s="28"/>
+      <c r="H99" s="28"/>
+      <c r="I99" s="28"/>
+      <c r="J99" s="28"/>
+      <c r="K99" s="28"/>
     </row>
     <row r="100" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="101" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -4684,46 +4710,46 @@
     <row r="122" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="123" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="124" spans="2:11" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C124" s="34" t="s">
+      <c r="C124" s="38" t="s">
         <v>246</v>
       </c>
-      <c r="D124" s="23"/>
-      <c r="E124" s="23"/>
-      <c r="F124" s="23"/>
-      <c r="G124" s="23"/>
-      <c r="H124" s="23"/>
-      <c r="I124" s="23"/>
-      <c r="J124" s="23"/>
-      <c r="K124" s="23"/>
+      <c r="D124" s="28"/>
+      <c r="E124" s="28"/>
+      <c r="F124" s="28"/>
+      <c r="G124" s="28"/>
+      <c r="H124" s="28"/>
+      <c r="I124" s="28"/>
+      <c r="J124" s="28"/>
+      <c r="K124" s="28"/>
     </row>
     <row r="126" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B126" s="21">
         <v>6</v>
       </c>
-      <c r="C126" s="33" t="s">
+      <c r="C126" s="39" t="s">
         <v>247</v>
       </c>
-      <c r="D126" s="23"/>
-      <c r="E126" s="23"/>
-      <c r="F126" s="23"/>
-      <c r="G126" s="23"/>
-      <c r="H126" s="23"/>
-      <c r="I126" s="23"/>
-      <c r="J126" s="23"/>
-      <c r="K126" s="23"/>
+      <c r="D126" s="28"/>
+      <c r="E126" s="28"/>
+      <c r="F126" s="28"/>
+      <c r="G126" s="28"/>
+      <c r="H126" s="28"/>
+      <c r="I126" s="28"/>
+      <c r="J126" s="28"/>
+      <c r="K126" s="28"/>
     </row>
     <row r="127" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C127" s="27" t="s">
+      <c r="C127" s="32" t="s">
         <v>248</v>
       </c>
-      <c r="D127" s="23"/>
-      <c r="E127" s="23"/>
-      <c r="F127" s="23"/>
-      <c r="G127" s="23"/>
-      <c r="H127" s="23"/>
-      <c r="I127" s="23"/>
-      <c r="J127" s="23"/>
-      <c r="K127" s="23"/>
+      <c r="D127" s="28"/>
+      <c r="E127" s="28"/>
+      <c r="F127" s="28"/>
+      <c r="G127" s="28"/>
+      <c r="H127" s="28"/>
+      <c r="I127" s="28"/>
+      <c r="J127" s="28"/>
+      <c r="K127" s="28"/>
     </row>
     <row r="128" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="129" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -4750,46 +4776,46 @@
     <row r="150" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="151" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="152" spans="2:11" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C152" s="34" t="s">
+      <c r="C152" s="38" t="s">
         <v>249</v>
       </c>
-      <c r="D152" s="23"/>
-      <c r="E152" s="23"/>
-      <c r="F152" s="23"/>
-      <c r="G152" s="23"/>
-      <c r="H152" s="23"/>
-      <c r="I152" s="23"/>
-      <c r="J152" s="23"/>
-      <c r="K152" s="23"/>
+      <c r="D152" s="28"/>
+      <c r="E152" s="28"/>
+      <c r="F152" s="28"/>
+      <c r="G152" s="28"/>
+      <c r="H152" s="28"/>
+      <c r="I152" s="28"/>
+      <c r="J152" s="28"/>
+      <c r="K152" s="28"/>
     </row>
     <row r="154" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B154" s="21">
         <v>7</v>
       </c>
-      <c r="C154" s="33" t="s">
+      <c r="C154" s="39" t="s">
         <v>250</v>
       </c>
-      <c r="D154" s="23"/>
-      <c r="E154" s="23"/>
-      <c r="F154" s="23"/>
-      <c r="G154" s="23"/>
-      <c r="H154" s="23"/>
-      <c r="I154" s="23"/>
-      <c r="J154" s="23"/>
-      <c r="K154" s="23"/>
+      <c r="D154" s="28"/>
+      <c r="E154" s="28"/>
+      <c r="F154" s="28"/>
+      <c r="G154" s="28"/>
+      <c r="H154" s="28"/>
+      <c r="I154" s="28"/>
+      <c r="J154" s="28"/>
+      <c r="K154" s="28"/>
     </row>
     <row r="155" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C155" s="27" t="s">
+      <c r="C155" s="32" t="s">
         <v>251</v>
       </c>
-      <c r="D155" s="23"/>
-      <c r="E155" s="23"/>
-      <c r="F155" s="23"/>
-      <c r="G155" s="23"/>
-      <c r="H155" s="23"/>
-      <c r="I155" s="23"/>
-      <c r="J155" s="23"/>
-      <c r="K155" s="23"/>
+      <c r="D155" s="28"/>
+      <c r="E155" s="28"/>
+      <c r="F155" s="28"/>
+      <c r="G155" s="28"/>
+      <c r="H155" s="28"/>
+      <c r="I155" s="28"/>
+      <c r="J155" s="28"/>
+      <c r="K155" s="28"/>
     </row>
     <row r="156" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="157" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -4807,46 +4833,46 @@
     <row r="169" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="170" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="171" spans="2:11" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C171" s="34" t="s">
+      <c r="C171" s="38" t="s">
         <v>252</v>
       </c>
-      <c r="D171" s="23"/>
-      <c r="E171" s="23"/>
-      <c r="F171" s="23"/>
-      <c r="G171" s="23"/>
-      <c r="H171" s="23"/>
-      <c r="I171" s="23"/>
-      <c r="J171" s="23"/>
-      <c r="K171" s="23"/>
+      <c r="D171" s="28"/>
+      <c r="E171" s="28"/>
+      <c r="F171" s="28"/>
+      <c r="G171" s="28"/>
+      <c r="H171" s="28"/>
+      <c r="I171" s="28"/>
+      <c r="J171" s="28"/>
+      <c r="K171" s="28"/>
     </row>
     <row r="173" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B173" s="21">
         <v>8</v>
       </c>
-      <c r="C173" s="33" t="s">
+      <c r="C173" s="39" t="s">
         <v>253</v>
       </c>
-      <c r="D173" s="23"/>
-      <c r="E173" s="23"/>
-      <c r="F173" s="23"/>
-      <c r="G173" s="23"/>
-      <c r="H173" s="23"/>
-      <c r="I173" s="23"/>
-      <c r="J173" s="23"/>
-      <c r="K173" s="23"/>
+      <c r="D173" s="28"/>
+      <c r="E173" s="28"/>
+      <c r="F173" s="28"/>
+      <c r="G173" s="28"/>
+      <c r="H173" s="28"/>
+      <c r="I173" s="28"/>
+      <c r="J173" s="28"/>
+      <c r="K173" s="28"/>
     </row>
     <row r="174" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C174" s="27" t="s">
+      <c r="C174" s="32" t="s">
         <v>254</v>
       </c>
-      <c r="D174" s="23"/>
-      <c r="E174" s="23"/>
-      <c r="F174" s="23"/>
-      <c r="G174" s="23"/>
-      <c r="H174" s="23"/>
-      <c r="I174" s="23"/>
-      <c r="J174" s="23"/>
-      <c r="K174" s="23"/>
+      <c r="D174" s="28"/>
+      <c r="E174" s="28"/>
+      <c r="F174" s="28"/>
+      <c r="G174" s="28"/>
+      <c r="H174" s="28"/>
+      <c r="I174" s="28"/>
+      <c r="J174" s="28"/>
+      <c r="K174" s="28"/>
     </row>
     <row r="175" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="176" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -4863,46 +4889,46 @@
     <row r="187" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="188" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="189" spans="2:11" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C189" s="34" t="s">
+      <c r="C189" s="38" t="s">
         <v>255</v>
       </c>
-      <c r="D189" s="23"/>
-      <c r="E189" s="23"/>
-      <c r="F189" s="23"/>
-      <c r="G189" s="23"/>
-      <c r="H189" s="23"/>
-      <c r="I189" s="23"/>
-      <c r="J189" s="23"/>
-      <c r="K189" s="23"/>
+      <c r="D189" s="28"/>
+      <c r="E189" s="28"/>
+      <c r="F189" s="28"/>
+      <c r="G189" s="28"/>
+      <c r="H189" s="28"/>
+      <c r="I189" s="28"/>
+      <c r="J189" s="28"/>
+      <c r="K189" s="28"/>
     </row>
     <row r="191" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B191" s="21">
         <v>9</v>
       </c>
-      <c r="C191" s="33" t="s">
+      <c r="C191" s="39" t="s">
         <v>256</v>
       </c>
-      <c r="D191" s="23"/>
-      <c r="E191" s="23"/>
-      <c r="F191" s="23"/>
-      <c r="G191" s="23"/>
-      <c r="H191" s="23"/>
-      <c r="I191" s="23"/>
-      <c r="J191" s="23"/>
-      <c r="K191" s="23"/>
+      <c r="D191" s="28"/>
+      <c r="E191" s="28"/>
+      <c r="F191" s="28"/>
+      <c r="G191" s="28"/>
+      <c r="H191" s="28"/>
+      <c r="I191" s="28"/>
+      <c r="J191" s="28"/>
+      <c r="K191" s="28"/>
     </row>
     <row r="192" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C192" s="27" t="s">
+      <c r="C192" s="32" t="s">
         <v>257</v>
       </c>
-      <c r="D192" s="23"/>
-      <c r="E192" s="23"/>
-      <c r="F192" s="23"/>
-      <c r="G192" s="23"/>
-      <c r="H192" s="23"/>
-      <c r="I192" s="23"/>
-      <c r="J192" s="23"/>
-      <c r="K192" s="23"/>
+      <c r="D192" s="28"/>
+      <c r="E192" s="28"/>
+      <c r="F192" s="28"/>
+      <c r="G192" s="28"/>
+      <c r="H192" s="28"/>
+      <c r="I192" s="28"/>
+      <c r="J192" s="28"/>
+      <c r="K192" s="28"/>
     </row>
     <row r="193" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="194" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -4929,46 +4955,46 @@
     <row r="215" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="216" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="217" spans="2:11" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C217" s="34" t="s">
+      <c r="C217" s="38" t="s">
         <v>258</v>
       </c>
-      <c r="D217" s="23"/>
-      <c r="E217" s="23"/>
-      <c r="F217" s="23"/>
-      <c r="G217" s="23"/>
-      <c r="H217" s="23"/>
-      <c r="I217" s="23"/>
-      <c r="J217" s="23"/>
-      <c r="K217" s="23"/>
+      <c r="D217" s="28"/>
+      <c r="E217" s="28"/>
+      <c r="F217" s="28"/>
+      <c r="G217" s="28"/>
+      <c r="H217" s="28"/>
+      <c r="I217" s="28"/>
+      <c r="J217" s="28"/>
+      <c r="K217" s="28"/>
     </row>
     <row r="219" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B219" s="21">
         <v>10</v>
       </c>
-      <c r="C219" s="33" t="s">
+      <c r="C219" s="39" t="s">
         <v>259</v>
       </c>
-      <c r="D219" s="23"/>
-      <c r="E219" s="23"/>
-      <c r="F219" s="23"/>
-      <c r="G219" s="23"/>
-      <c r="H219" s="23"/>
-      <c r="I219" s="23"/>
-      <c r="J219" s="23"/>
-      <c r="K219" s="23"/>
+      <c r="D219" s="28"/>
+      <c r="E219" s="28"/>
+      <c r="F219" s="28"/>
+      <c r="G219" s="28"/>
+      <c r="H219" s="28"/>
+      <c r="I219" s="28"/>
+      <c r="J219" s="28"/>
+      <c r="K219" s="28"/>
     </row>
     <row r="220" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C220" s="27" t="s">
+      <c r="C220" s="32" t="s">
         <v>260</v>
       </c>
-      <c r="D220" s="23"/>
-      <c r="E220" s="23"/>
-      <c r="F220" s="23"/>
-      <c r="G220" s="23"/>
-      <c r="H220" s="23"/>
-      <c r="I220" s="23"/>
-      <c r="J220" s="23"/>
-      <c r="K220" s="23"/>
+      <c r="D220" s="28"/>
+      <c r="E220" s="28"/>
+      <c r="F220" s="28"/>
+      <c r="G220" s="28"/>
+      <c r="H220" s="28"/>
+      <c r="I220" s="28"/>
+      <c r="J220" s="28"/>
+      <c r="K220" s="28"/>
     </row>
     <row r="221" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="222" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -4989,58 +5015,58 @@
     <row r="237" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="238" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="239" spans="3:11" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C239" s="34" t="s">
+      <c r="C239" s="38" t="s">
         <v>261</v>
       </c>
-      <c r="D239" s="23"/>
-      <c r="E239" s="23"/>
-      <c r="F239" s="23"/>
-      <c r="G239" s="23"/>
-      <c r="H239" s="23"/>
-      <c r="I239" s="23"/>
-      <c r="J239" s="23"/>
-      <c r="K239" s="23"/>
+      <c r="D239" s="28"/>
+      <c r="E239" s="28"/>
+      <c r="F239" s="28"/>
+      <c r="G239" s="28"/>
+      <c r="H239" s="28"/>
+      <c r="I239" s="28"/>
+      <c r="J239" s="28"/>
+      <c r="K239" s="28"/>
     </row>
     <row r="241" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A241" s="28" t="s">
+      <c r="A241" s="33" t="s">
         <v>262</v>
       </c>
-      <c r="B241" s="23"/>
-      <c r="C241" s="23"/>
-      <c r="D241" s="23"/>
-      <c r="E241" s="23"/>
-      <c r="F241" s="23"/>
-      <c r="G241" s="23"/>
-      <c r="H241" s="23"/>
-      <c r="I241" s="23"/>
-      <c r="J241" s="23"/>
-      <c r="K241" s="23"/>
+      <c r="B241" s="28"/>
+      <c r="C241" s="28"/>
+      <c r="D241" s="28"/>
+      <c r="E241" s="28"/>
+      <c r="F241" s="28"/>
+      <c r="G241" s="28"/>
+      <c r="H241" s="28"/>
+      <c r="I241" s="28"/>
+      <c r="J241" s="28"/>
+      <c r="K241" s="28"/>
     </row>
     <row r="242" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C242" s="33" t="s">
+      <c r="C242" s="39" t="s">
         <v>263</v>
       </c>
-      <c r="D242" s="23"/>
-      <c r="E242" s="23"/>
-      <c r="F242" s="23"/>
-      <c r="G242" s="23"/>
-      <c r="H242" s="23"/>
-      <c r="I242" s="23"/>
-      <c r="J242" s="23"/>
-      <c r="K242" s="23"/>
+      <c r="D242" s="28"/>
+      <c r="E242" s="28"/>
+      <c r="F242" s="28"/>
+      <c r="G242" s="28"/>
+      <c r="H242" s="28"/>
+      <c r="I242" s="28"/>
+      <c r="J242" s="28"/>
+      <c r="K242" s="28"/>
     </row>
     <row r="243" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C243" s="27" t="s">
+      <c r="C243" s="32" t="s">
         <v>264</v>
       </c>
-      <c r="D243" s="23"/>
-      <c r="E243" s="23"/>
-      <c r="F243" s="23"/>
-      <c r="G243" s="23"/>
-      <c r="H243" s="23"/>
-      <c r="I243" s="23"/>
-      <c r="J243" s="23"/>
-      <c r="K243" s="23"/>
+      <c r="D243" s="28"/>
+      <c r="E243" s="28"/>
+      <c r="F243" s="28"/>
+      <c r="G243" s="28"/>
+      <c r="H243" s="28"/>
+      <c r="I243" s="28"/>
+      <c r="J243" s="28"/>
+      <c r="K243" s="28"/>
     </row>
     <row r="244" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="245" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -5067,43 +5093,43 @@
     <row r="266" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="267" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="268" spans="3:11" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C268" s="34" t="s">
+      <c r="C268" s="38" t="s">
         <v>265</v>
       </c>
-      <c r="D268" s="23"/>
-      <c r="E268" s="23"/>
-      <c r="F268" s="23"/>
-      <c r="G268" s="23"/>
-      <c r="H268" s="23"/>
-      <c r="I268" s="23"/>
-      <c r="J268" s="23"/>
-      <c r="K268" s="23"/>
+      <c r="D268" s="28"/>
+      <c r="E268" s="28"/>
+      <c r="F268" s="28"/>
+      <c r="G268" s="28"/>
+      <c r="H268" s="28"/>
+      <c r="I268" s="28"/>
+      <c r="J268" s="28"/>
+      <c r="K268" s="28"/>
     </row>
     <row r="270" spans="3:11" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C270" s="33" t="s">
+      <c r="C270" s="39" t="s">
         <v>266</v>
       </c>
-      <c r="D270" s="23"/>
-      <c r="E270" s="23"/>
-      <c r="F270" s="23"/>
-      <c r="G270" s="23"/>
-      <c r="H270" s="23"/>
-      <c r="I270" s="23"/>
-      <c r="J270" s="23"/>
-      <c r="K270" s="23"/>
+      <c r="D270" s="28"/>
+      <c r="E270" s="28"/>
+      <c r="F270" s="28"/>
+      <c r="G270" s="28"/>
+      <c r="H270" s="28"/>
+      <c r="I270" s="28"/>
+      <c r="J270" s="28"/>
+      <c r="K270" s="28"/>
     </row>
     <row r="271" spans="3:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C271" s="27" t="s">
+      <c r="C271" s="32" t="s">
         <v>267</v>
       </c>
-      <c r="D271" s="23"/>
-      <c r="E271" s="23"/>
-      <c r="F271" s="23"/>
-      <c r="G271" s="23"/>
-      <c r="H271" s="23"/>
-      <c r="I271" s="23"/>
-      <c r="J271" s="23"/>
-      <c r="K271" s="23"/>
+      <c r="D271" s="28"/>
+      <c r="E271" s="28"/>
+      <c r="F271" s="28"/>
+      <c r="G271" s="28"/>
+      <c r="H271" s="28"/>
+      <c r="I271" s="28"/>
+      <c r="J271" s="28"/>
+      <c r="K271" s="28"/>
     </row>
     <row r="272" spans="3:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="273" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -5126,157 +5152,143 @@
     <row r="290" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="291" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="292" spans="1:11" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C292" s="34" t="s">
+      <c r="C292" s="38" t="s">
         <v>268</v>
       </c>
-      <c r="D292" s="23"/>
-      <c r="E292" s="23"/>
-      <c r="F292" s="23"/>
-      <c r="G292" s="23"/>
-      <c r="H292" s="23"/>
-      <c r="I292" s="23"/>
-      <c r="J292" s="23"/>
-      <c r="K292" s="23"/>
+      <c r="D292" s="28"/>
+      <c r="E292" s="28"/>
+      <c r="F292" s="28"/>
+      <c r="G292" s="28"/>
+      <c r="H292" s="28"/>
+      <c r="I292" s="28"/>
+      <c r="J292" s="28"/>
+      <c r="K292" s="28"/>
     </row>
     <row r="294" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A294" s="28" t="s">
+      <c r="A294" s="33" t="s">
         <v>269</v>
       </c>
-      <c r="B294" s="23"/>
-      <c r="C294" s="23"/>
-      <c r="D294" s="23"/>
-      <c r="E294" s="23"/>
-      <c r="F294" s="23"/>
-      <c r="G294" s="23"/>
-      <c r="H294" s="23"/>
-      <c r="I294" s="23"/>
-      <c r="J294" s="23"/>
-      <c r="K294" s="23"/>
+      <c r="B294" s="28"/>
+      <c r="C294" s="28"/>
+      <c r="D294" s="28"/>
+      <c r="E294" s="28"/>
+      <c r="F294" s="28"/>
+      <c r="G294" s="28"/>
+      <c r="H294" s="28"/>
+      <c r="I294" s="28"/>
+      <c r="J294" s="28"/>
+      <c r="K294" s="28"/>
     </row>
     <row r="295" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B295" s="27" t="s">
+      <c r="B295" s="32" t="s">
         <v>270</v>
       </c>
-      <c r="C295" s="23"/>
-      <c r="D295" s="23"/>
-      <c r="E295" s="23"/>
-      <c r="F295" s="23"/>
-      <c r="G295" s="23"/>
-      <c r="H295" s="23"/>
-      <c r="I295" s="23"/>
-      <c r="J295" s="23"/>
-      <c r="K295" s="23"/>
+      <c r="C295" s="28"/>
+      <c r="D295" s="28"/>
+      <c r="E295" s="28"/>
+      <c r="F295" s="28"/>
+      <c r="G295" s="28"/>
+      <c r="H295" s="28"/>
+      <c r="I295" s="28"/>
+      <c r="J295" s="28"/>
+      <c r="K295" s="28"/>
     </row>
     <row r="296" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B296" s="27" t="s">
+      <c r="B296" s="32" t="s">
         <v>271</v>
       </c>
-      <c r="C296" s="23"/>
-      <c r="D296" s="23"/>
-      <c r="E296" s="23"/>
-      <c r="F296" s="23"/>
-      <c r="G296" s="23"/>
-      <c r="H296" s="23"/>
-      <c r="I296" s="23"/>
-      <c r="J296" s="23"/>
-      <c r="K296" s="23"/>
+      <c r="C296" s="28"/>
+      <c r="D296" s="28"/>
+      <c r="E296" s="28"/>
+      <c r="F296" s="28"/>
+      <c r="G296" s="28"/>
+      <c r="H296" s="28"/>
+      <c r="I296" s="28"/>
+      <c r="J296" s="28"/>
+      <c r="K296" s="28"/>
     </row>
     <row r="297" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B297" s="27" t="s">
+      <c r="B297" s="32" t="s">
         <v>272</v>
       </c>
-      <c r="C297" s="23"/>
-      <c r="D297" s="23"/>
-      <c r="E297" s="23"/>
-      <c r="F297" s="23"/>
-      <c r="G297" s="23"/>
-      <c r="H297" s="23"/>
-      <c r="I297" s="23"/>
-      <c r="J297" s="23"/>
-      <c r="K297" s="23"/>
+      <c r="C297" s="28"/>
+      <c r="D297" s="28"/>
+      <c r="E297" s="28"/>
+      <c r="F297" s="28"/>
+      <c r="G297" s="28"/>
+      <c r="H297" s="28"/>
+      <c r="I297" s="28"/>
+      <c r="J297" s="28"/>
+      <c r="K297" s="28"/>
     </row>
     <row r="298" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B298" s="27" t="s">
+      <c r="B298" s="32" t="s">
         <v>273</v>
       </c>
-      <c r="C298" s="23"/>
-      <c r="D298" s="23"/>
-      <c r="E298" s="23"/>
-      <c r="F298" s="23"/>
-      <c r="G298" s="23"/>
-      <c r="H298" s="23"/>
-      <c r="I298" s="23"/>
-      <c r="J298" s="23"/>
-      <c r="K298" s="23"/>
+      <c r="C298" s="28"/>
+      <c r="D298" s="28"/>
+      <c r="E298" s="28"/>
+      <c r="F298" s="28"/>
+      <c r="G298" s="28"/>
+      <c r="H298" s="28"/>
+      <c r="I298" s="28"/>
+      <c r="J298" s="28"/>
+      <c r="K298" s="28"/>
     </row>
     <row r="299" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B299" s="27" t="s">
+      <c r="B299" s="32" t="s">
         <v>274</v>
       </c>
-      <c r="C299" s="23"/>
-      <c r="D299" s="23"/>
-      <c r="E299" s="23"/>
-      <c r="F299" s="23"/>
-      <c r="G299" s="23"/>
-      <c r="H299" s="23"/>
-      <c r="I299" s="23"/>
-      <c r="J299" s="23"/>
-      <c r="K299" s="23"/>
+      <c r="C299" s="28"/>
+      <c r="D299" s="28"/>
+      <c r="E299" s="28"/>
+      <c r="F299" s="28"/>
+      <c r="G299" s="28"/>
+      <c r="H299" s="28"/>
+      <c r="I299" s="28"/>
+      <c r="J299" s="28"/>
+      <c r="K299" s="28"/>
     </row>
     <row r="301" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A301" s="40" t="s">
         <v>275</v>
       </c>
-      <c r="B301" s="23"/>
-      <c r="C301" s="23"/>
-      <c r="D301" s="23"/>
-      <c r="E301" s="23"/>
-      <c r="F301" s="23"/>
-      <c r="G301" s="23"/>
-      <c r="H301" s="23"/>
-      <c r="I301" s="23"/>
-      <c r="J301" s="23"/>
-      <c r="K301" s="23"/>
+      <c r="B301" s="28"/>
+      <c r="C301" s="28"/>
+      <c r="D301" s="28"/>
+      <c r="E301" s="28"/>
+      <c r="F301" s="28"/>
+      <c r="G301" s="28"/>
+      <c r="H301" s="28"/>
+      <c r="I301" s="28"/>
+      <c r="J301" s="28"/>
+      <c r="K301" s="28"/>
     </row>
     <row r="302" spans="1:11" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A302" s="32" t="s">
-        <v>276</v>
-      </c>
-      <c r="B302" s="23"/>
-      <c r="C302" s="23"/>
-      <c r="D302" s="23"/>
-      <c r="E302" s="23"/>
-      <c r="F302" s="23"/>
-      <c r="G302" s="23"/>
-      <c r="H302" s="23"/>
-      <c r="I302" s="23"/>
-      <c r="J302" s="23"/>
-      <c r="K302" s="23"/>
+      <c r="A302" s="34" t="s">
+        <v>284</v>
+      </c>
+      <c r="B302" s="28"/>
+      <c r="C302" s="28"/>
+      <c r="D302" s="28"/>
+      <c r="E302" s="28"/>
+      <c r="F302" s="28"/>
+      <c r="G302" s="28"/>
+      <c r="H302" s="28"/>
+      <c r="I302" s="28"/>
+      <c r="J302" s="28"/>
+      <c r="K302" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="A302:K302"/>
-    <mergeCell ref="C220:K220"/>
-    <mergeCell ref="C239:K239"/>
-    <mergeCell ref="C68:K68"/>
-    <mergeCell ref="C98:K98"/>
-    <mergeCell ref="C191:K191"/>
-    <mergeCell ref="B299:K299"/>
-    <mergeCell ref="C126:K126"/>
-    <mergeCell ref="C171:K171"/>
-    <mergeCell ref="A301:K301"/>
-    <mergeCell ref="C155:K155"/>
-    <mergeCell ref="C217:K217"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="C189:K189"/>
-    <mergeCell ref="C96:K96"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="B297:K297"/>
-    <mergeCell ref="C154:K154"/>
-    <mergeCell ref="C42:K42"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C20:K20"/>
-    <mergeCell ref="A9:K9"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="C242:K242"/>
+    <mergeCell ref="C192:K192"/>
+    <mergeCell ref="C43:K43"/>
+    <mergeCell ref="C16:K16"/>
+    <mergeCell ref="C271:K271"/>
+    <mergeCell ref="C152:K152"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A241:K241"/>
     <mergeCell ref="C71:K71"/>
@@ -5292,25 +5304,39 @@
     <mergeCell ref="C19:K19"/>
     <mergeCell ref="C292:K292"/>
     <mergeCell ref="A294:K294"/>
-    <mergeCell ref="B298:K298"/>
     <mergeCell ref="A3:K4"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="C189:K189"/>
+    <mergeCell ref="C96:K96"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="B297:K297"/>
+    <mergeCell ref="C154:K154"/>
+    <mergeCell ref="C42:K42"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C20:K20"/>
+    <mergeCell ref="A9:K9"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="C99:K99"/>
     <mergeCell ref="C270:K270"/>
     <mergeCell ref="H12:K12"/>
     <mergeCell ref="C40:K40"/>
     <mergeCell ref="A11:K11"/>
+    <mergeCell ref="A302:K302"/>
+    <mergeCell ref="C220:K220"/>
+    <mergeCell ref="C239:K239"/>
+    <mergeCell ref="C68:K68"/>
+    <mergeCell ref="C98:K98"/>
+    <mergeCell ref="C191:K191"/>
+    <mergeCell ref="B299:K299"/>
+    <mergeCell ref="C126:K126"/>
+    <mergeCell ref="C171:K171"/>
+    <mergeCell ref="A301:K301"/>
+    <mergeCell ref="C155:K155"/>
+    <mergeCell ref="C217:K217"/>
+    <mergeCell ref="B298:K298"/>
     <mergeCell ref="C124:K124"/>
     <mergeCell ref="C127:K127"/>
     <mergeCell ref="C173:K173"/>
-    <mergeCell ref="C242:K242"/>
-    <mergeCell ref="C192:K192"/>
-    <mergeCell ref="C43:K43"/>
-    <mergeCell ref="C16:K16"/>
-    <mergeCell ref="C271:K271"/>
-    <mergeCell ref="C152:K152"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="E13:G13"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H12" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>

</xml_diff>

<commit_message>
Templates: remove saved folder location and last-modified-by name from workbook metadata
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finance-controlling/ABZON-asset-acquisition.xlsx
+++ b/finance-controlling/ABZON-asset-acquisition.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24a7865e3124cb3d/Documents/PostNow/github-templates/finance-controlling/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="28" documentId="11_C5ADC2FD48FB3D1BDA0814AFE865F60D2B8650A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83B22C3D-9B4C-4635-901F-AFDED2F4F770}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>

</xml_diff>